<commit_message>
update soal soal KMSI
</commit_message>
<xml_diff>
--- a/docs/blueprint/menu-belajar.xlsx
+++ b/docs/blueprint/menu-belajar.xlsx
@@ -550,7 +550,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Menu Belajar Udakids: Pra-TK, TK, Kelas 1</t>
+          <t>Menu Belajar Udakids: PAUD, TK, Kelas 1</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Fase G4 = Pra-TK, G5 = TK, G6 = Kelas 1. Kerjakan berurutan dari kode terkecil (unit awal jadi dasar unit berikutnya).</t>
+          <t>• Fase G4 = PAUD, G5 = TK, G6 = Kelas 1. Kerjakan berurutan dari kode terkecil (unit awal jadi dasar unit berikutnya).</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -906,7 +906,7 @@
       <c r="S2" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-01 · Pra-TK · Baca Tulis · Dengar bunyi di sekitarku
+UNIT P-BT-01 · PAUD · Baca Tulis · Dengar bunyi di sekitarku
 Tujuan: Membedakan bunyi hewan, kendaraan, dan benda. Rujukan: CP Fondasi literasi; L&amp;S Phase 1.
 Tema kosakata: hewan, kendaraan, alat musik. Model latihan: 1, 14. Layar pelajaran: bunyi, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -917,7 +917,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -931,7 +931,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -1005,7 +1005,7 @@
       <c r="S3" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-02 · Pra-TK · Baca Tulis · Garis tegak dan mendatar
+UNIT P-BT-02 · PAUD · Baca Tulis · Garis tegak dan mendatar
 Tujuan: Kontrol gerak jari sebelum menulis huruf. Rujukan: CP Fondasi motorik.
 Tema kosakata: benda sekitar. Model latihan: 10, 19. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1016,7 +1016,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -1104,7 +1104,7 @@
       <c r="S4" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-03 · Pra-TK · Baca Tulis · Garis lengkung, lingkaran, zig-zag
+UNIT P-BT-03 · PAUD · Baca Tulis · Garis lengkung, lingkaran, zig-zag
 Tujuan: Pola goresan dasar huruf. Rujukan: CP Fondasi motorik.
 Tema kosakata: alam (ombak, gunung). Model latihan: 10, 19. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1115,7 +1115,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Pelajaran baru + soal baru</t>
+          <t>Draf (Worksheet PAUD C)</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
@@ -1203,7 +1203,7 @@
       <c r="S5" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-04 · Pra-TK · Baca Tulis · Huruf vokal a dan i
+UNIT P-BT-04 · PAUD · Baca Tulis · Huruf vokal a dan i
 Tujuan: Mengenal bentuk dan bunyi a, i. Rujukan: CP Fondasi literasi; metode suku kata.
 Tema kosakata: buah, hewan. Model latihan: 2, 8, 10. Layar pelajaran: kenalan, bunyi, kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1214,7 +1214,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>Pelajaran baru + soal baru</t>
+          <t>Draf (Worksheet PAUD D)</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -1302,7 +1302,7 @@
       <c r="S6" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-05 · Pra-TK · Baca Tulis · Huruf vokal u, e, o
+UNIT P-BT-05 · PAUD · Baca Tulis · Huruf vokal u, e, o
 Tujuan: Mengenal bentuk dan bunyi u, e, o. Rujukan: CP Fondasi literasi.
 Tema kosakata: benda rumah, alam. Model latihan: 2, 8, 10. Layar pelajaran: kenalan, bunyi, kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1313,7 +1313,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1401,7 +1401,7 @@
       <c r="S7" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-06 · Pra-TK · Baca Tulis · Huruf awal benda (vokal)
+UNIT P-BT-06 · PAUD · Baca Tulis · Huruf awal benda (vokal)
 Tujuan: Menghubungkan gambar dengan huruf awalnya. Rujukan: CP Fondasi literasi.
 Tema kosakata: semua tema T1. Model latihan: 8, 1, 14. Layar pelajaran: kata, ingat.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1412,7 +1412,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1500,7 +1500,7 @@
       <c r="S8" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-07 · Pra-TK · Baca Tulis · Tepuk suku kata
+UNIT P-BT-07 · PAUD · Baca Tulis · Tepuk suku kata
 Tujuan: Menyadari kata terdiri dari suku kata (ba-ju). Rujukan: Metode suku kata; L&amp;S Phase 1.
 Tema kosakata: pakaian, makanan. Model latihan: 1, 3. Layar pelajaran: bunyi, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1511,7 +1511,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1599,7 +1599,7 @@
       <c r="S9" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-08 · Pra-TK · Baca Tulis · Bunyi akhir yang sama (rima)
+UNIT P-BT-08 · PAUD · Baca Tulis · Bunyi akhir yang sama (rima)
 Tujuan: Mendengar kata berakhiran sama (topi-kopi). Rujukan: L&amp;S Phase 1.
 Tema kosakata: benda sekitar. Model latihan: 1, 14. Layar pelajaran: bunyi, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1610,7 +1610,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1698,7 +1698,7 @@
       <c r="S10" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-09 · Pra-TK · Baca Tulis · Huruf bibir: b, m, p
+UNIT P-BT-09 · PAUD · Baca Tulis · Huruf bibir: b, m, p
 Tujuan: Mengenal konsonan pertama yang mudah dilafalkan. Rujukan: Metode suku kata.
 Tema kosakata: hewan, mainan. Model latihan: 2, 8, 10. Layar pelajaran: kenalan, bunyi, kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1709,7 +1709,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1797,7 +1797,7 @@
       <c r="S11" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-10 · Pra-TK · Baca Tulis · Cerita bergambar
+UNIT P-BT-10 · PAUD · Baca Tulis · Cerita bergambar
 Tujuan: Mengurutkan 3 gambar dan menceritakannya. Rujukan: CP Fondasi literasi; NEL L&amp;L.
 Tema kosakata: kegiatan sehari-hari. Model latihan: 6, 24. Layar pelajaran: cerita, ingat.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1808,7 +1808,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1896,7 +1896,7 @@
       <c r="S12" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-BT-11 · Pra-TK · Baca Tulis · 100 kata pertamaku
+UNIT P-BT-11 · PAUD · Baca Tulis · 100 kata pertamaku
 Tujuan: Kosakata benda paling dekat dengan anak. Rujukan: CDI / Biemiller.
 Tema kosakata: Kamus T1 (100 kata). Model latihan: 1, 14, 15. Layar pelajaran: kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -1907,7 +1907,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Bilangan 1 sampai 5</t>
+          <t>Bilangan 1 sampai 10</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Membilang dan mengenal lambang 1–5</t>
+          <t>Membilang dan mengenal lambang 1–10</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Ada: Math Pra-TK A, B, C, D</t>
+          <t>Ada: Worksheet Pra-TK A; Math Pra-TK A, B, C, D</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>Pelajaran baru + soal sudah ada</t>
+          <t>Draf (Worksheet PAUD A)</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -1995,8 +1995,8 @@
       <c r="S13" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-01 · Pra-TK · Berhitung · Bilangan 1 sampai 5
-Tujuan: Membilang dan mengenal lambang 1–5. Rujukan: CP Fondasi; NEL; EYFS.
+UNIT P-MA-01 · PAUD · Berhitung · Bilangan 1 sampai 10
+Tujuan: Membilang dan mengenal lambang 1–10. Rujukan: CP Fondasi; NEL; EYFS.
 Tema kosakata: buah, hewan, mainan. Model latihan: 3, 4, 8. Layar pelajaran: kenalan, kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
 semua teks bisa dibacakan; maksimal 4 pilihan; tanpa kata "salah/gagal"; pujian menyebut usaha; tanpa batas waktu;
@@ -2006,7 +2006,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): tidak perlu. Tantangan memakai buku yang sudah ada (Math Pra-TK A, B, C, D).
+BAGIAN B (soal): tidak perlu. Tantangan memakai buku yang sudah ada (Worksheet Pra-TK A; Math Pra-TK A, B, C, D).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -2094,7 +2094,7 @@
       <c r="S14" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-02 · Pra-TK · Berhitung · Lihat sekilas 1 sampai 5
+UNIT P-MA-02 · PAUD · Berhitung · Lihat sekilas 1 sampai 5
 Tujuan: Mengenali banyak benda tanpa menghitung satu-satu. Rujukan: EYFS Number (subitising).
 Tema kosakata: titik, buah. Model latihan: 16, 3. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2105,7 +2105,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -2193,7 +2193,7 @@
       <c r="S15" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-03 · Pra-TK · Berhitung · Bilangan 6 sampai 10
+UNIT P-MA-03 · PAUD · Berhitung · Bilangan 6 sampai 10
 Tujuan: Membilang dan mengenal lambang 6–10. Rujukan: CP Fondasi; NEL.
 Tema kosakata: makanan, kendaraan. Model latihan: 3, 4, 5. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2218,7 +2218,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -2292,7 +2292,7 @@
       <c r="S16" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-04 · Pra-TK · Berhitung · Jari tangan dan angka
+UNIT P-MA-04 · PAUD · Berhitung · Jari tangan dan angka
 Tujuan: Menunjukkan bilangan dengan jari. Rujukan: NEL Numeracy.
 Tema kosakata: tubuh (jari). Model latihan: 8, 16. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2303,7 +2303,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -2391,7 +2391,7 @@
       <c r="S17" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-05 · Pra-TK · Berhitung · Pertama sampai kelima
+UNIT P-MA-05 · PAUD · Berhitung · Pertama sampai kelima
 Tujuan: Bilangan urutan dalam antrean. Rujukan: Common Core K.CC; NEL.
 Tema kosakata: hewan, kendaraan. Model latihan: 13, 6. Layar pelajaran: cerita, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2402,7 +2402,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -2490,7 +2490,7 @@
       <c r="S18" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-06 · Pra-TK · Berhitung · Lebih banyak, lebih sedikit
+UNIT P-MA-06 · PAUD · Berhitung · Lebih banyak, lebih sedikit
 Tujuan: Membandingkan dua kelompok. Rujukan: CP Fondasi; EYFS.
 Tema kosakata: buah, mainan. Model latihan: 1, 4. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2515,7 +2515,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -2589,7 +2589,7 @@
       <c r="S19" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-07 · Pra-TK · Berhitung · Pola warna dan bentuk
+UNIT P-MA-07 · PAUD · Berhitung · Pola warna dan bentuk
 Tujuan: Melanjutkan pola AB, AAB. Rujukan: CP Fondasi (pola); NEL.
 Tema kosakata: warna, bentuk. Model latihan: 20, 6. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
@@ -2688,7 +2688,7 @@
       <c r="S20" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-08 · Pra-TK · Berhitung · Di atas, di bawah, di dalam
+UNIT P-MA-08 · PAUD · Berhitung · Di atas, di bawah, di dalam
 Tujuan: Kata posisi. Rujukan: NEL bentuk &amp; ruang.
 Tema kosakata: rumah, mainan. Model latihan: 13, 1. Layar pelajaran: cerita, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2713,7 +2713,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -2787,7 +2787,7 @@
       <c r="S21" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-09 · Pra-TK · Berhitung · Bentuk di sekitarku
+UNIT P-MA-09 · PAUD · Berhitung · Bentuk di sekitarku
 Tujuan: Mengenal lingkaran, segitiga, persegi, bangun ruang. Rujukan: CP Fondasi; Common Core K.G.
 Tema kosakata: benda rumah. Model latihan: 1, 7, 15. Layar pelajaran: kenalan, kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2812,7 +2812,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -2886,7 +2886,7 @@
       <c r="S22" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-10 · Pra-TK · Berhitung · Besar-kecil, panjang-pendek
+UNIT P-MA-10 · PAUD · Berhitung · Besar-kecil, panjang-pendek
 Tujuan: Membandingkan ukuran. Rujukan: CP Fondasi (ukur).
 Tema kosakata: hewan, benda. Model latihan: 6, 17. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -2911,7 +2911,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -2985,7 +2985,7 @@
       <c r="S23" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-11 · Pra-TK · Berhitung · Sama, beda, kelompokkan
+UNIT P-MA-11 · PAUD · Berhitung · Sama, beda, kelompokkan
 Tujuan: Mengklasifikasi benda. Rujukan: CP Fondasi (klasifikasi).
 Tema kosakata: semua tema T1. Model latihan: 7, 15. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3010,7 +3010,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -3084,7 +3084,7 @@
       <c r="S24" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-12 · Pra-TK · Berhitung · Tambah dan kurang sampai 5
+UNIT P-MA-12 · PAUD · Berhitung · Tambah dan kurang sampai 5
 Tujuan: Menggabung dan mengambil benda. Rujukan: EYFS; Common Core K.OA.
 Tema kosakata: makanan, hewan. Model latihan: 3, 4, 18. Layar pelajaran: cerita, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -3183,7 +3183,7 @@
       <c r="S25" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-13 · Pra-TK · Berhitung · Uang Rupiah
+UNIT P-MA-13 · PAUD · Berhitung · Uang Rupiah
 Tujuan: Mengenal koin dan uang kertas. Rujukan: Konteks lokal.
 Tema kosakata: pasar, jajanan. Model latihan: 1, 7. Layar pelajaran: kenalan, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -3282,7 +3282,7 @@
       <c r="S26" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-MA-14 · Pra-TK · Berhitung · Pagi, siang, malam
+UNIT P-MA-14 · PAUD · Berhitung · Pagi, siang, malam
 Tujuan: Kesadaran waktu dalam kegiatan. Rujukan: CP Fondasi (waktu).
 Tema kosakata: kegiatan sehari-hari, langit. Model latihan: 6, 1. Layar pelajaran: cerita, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3293,7 +3293,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -3381,7 +3381,7 @@
       <c r="S27" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-01 · Pra-TK · English · Hello! Greetings &amp; feelings
+UNIT P-EN-01 · PAUD · English · Hello! Greetings &amp; feelings
 Tujuan: Salam dan perasaan sederhana. Rujukan: Cambridge Pre A1 Starters.
 Tema kosakata: perasaan. Model latihan: 1, 21. Layar pelajaran: kata, bunyi.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3392,7 +3392,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -3480,7 +3480,7 @@
       <c r="S28" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-02 · Pra-TK · English · Letters A–Z
+UNIT P-EN-02 · PAUD · English · Letters A–Z
 Tujuan: Nama huruf A–Z. Rujukan: NEL L&amp;L; Starters.
 Tema kosakata: kata contoh A–Z. Model latihan: 2, 8. Layar pelajaran: kenalan, bunyi.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3505,7 +3505,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -3579,7 +3579,7 @@
       <c r="S29" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-03 · Pra-TK · English · Big and small letters
+UNIT P-EN-03 · PAUD · English · Big and small letters
 Tujuan: Huruf besar dan kecil. Rujukan: NEL L&amp;L.
 Tema kosakata: kata contoh. Model latihan: 8, 10. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3604,7 +3604,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -3678,7 +3678,7 @@
       <c r="S30" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-04 · Pra-TK · English · Sounds around me
+UNIT P-EN-04 · PAUD · English · Sounds around me
 Tujuan: Bunyi awal kata. Rujukan: L&amp;S Phase 1–2.
 Tema kosakata: hewan, makanan. Model latihan: 1, 8. Layar pelajaran: bunyi, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3703,7 +3703,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -3777,7 +3777,7 @@
       <c r="S31" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-05 · Pra-TK · English · Rhymes and syllables
+UNIT P-EN-05 · PAUD · English · Rhymes and syllables
 Tujuan: Rima dan suku kata. Rujukan: L&amp;S Phase 1.
 Tema kosakata: benda. Model latihan: 1, 14. Layar pelajaran: bunyi, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3802,7 +3802,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -3876,7 +3876,7 @@
       <c r="S32" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-06 · Pra-TK · English · Colours and shapes
+UNIT P-EN-06 · PAUD · English · Colours and shapes
 Tujuan: Kata warna dan bentuk. Rujukan: Starters.
 Tema kosakata: warna, bentuk. Model latihan: 1, 7. Layar pelajaran: kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -3975,7 +3975,7 @@
       <c r="S33" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-07 · Pra-TK · English · Numbers 1–10
+UNIT P-EN-07 · PAUD · English · Numbers 1–10
 Tujuan: Kata bilangan. Rujukan: Starters.
 Tema kosakata: buah, mainan. Model latihan: 3, 8. Layar pelajaran: kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4000,7 +4000,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
@@ -4074,7 +4074,7 @@
       <c r="S34" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-08 · Pra-TK · English · My body
+UNIT P-EN-08 · PAUD · English · My body
 Tujuan: Anggota tubuh. Rujukan: Starters (body &amp; face).
 Tema kosakata: tubuh. Model latihan: 1, 13. Layar pelajaran: kata, cerita.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4085,7 +4085,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
@@ -4173,7 +4173,7 @@
       <c r="S35" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-09 · Pra-TK · English · Animals
+UNIT P-EN-09 · PAUD · English · Animals
 Tujuan: Hewan. Rujukan: Starters (animals).
 Tema kosakata: hewan. Model latihan: 1, 14, 7. Layar pelajaran: kata, bunyi.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4184,7 +4184,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
@@ -4272,7 +4272,7 @@
       <c r="S36" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-10 · Pra-TK · English · Food and fruit
+UNIT P-EN-10 · PAUD · English · Food and fruit
 Tujuan: Makanan dan buah. Rujukan: Starters (food &amp; drink).
 Tema kosakata: buah, makanan. Model latihan: 1, 7, 14. Layar pelajaran: kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4283,7 +4283,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -4371,7 +4371,7 @@
       <c r="S37" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-11 · Pra-TK · English · Action words
+UNIT P-EN-11 · PAUD · English · Action words
 Tujuan: Kata kerja. Rujukan: Starters.
 Tema kosakata: kegiatan. Model latihan: 1, 13. Layar pelajaran: kata, cerita.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4396,7 +4396,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
@@ -4470,7 +4470,7 @@
       <c r="S38" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-12 · Pra-TK · English · In, on, under
+UNIT P-EN-12 · PAUD · English · In, on, under
 Tujuan: Kata posisi. Rujukan: Starters (prepositions).
 Tema kosakata: rumah, mainan. Model latihan: 23, 13. Layar pelajaran: cerita, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4495,7 +4495,7 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
@@ -4569,7 +4569,7 @@
       <c r="S39" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-EN-13 · Pra-TK · English · Opposites and categories
+UNIT P-EN-13 · PAUD · English · Opposites and categories
 Tujuan: Lawan kata dan kelompok. Rujukan: Starters; NEL.
 Tema kosakata: semua tema. Model latihan: 7, 15. Layar pelajaran: kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4594,7 +4594,7 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -4668,7 +4668,7 @@
       <c r="S40" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-01 · Pra-TK · Sains · Tubuhku dan panca indra
+UNIT P-SA-01 · PAUD · Sains · Tubuhku dan panca indra
 Tujuan: Mata melihat, telinga mendengar, dst.. Rujukan: CP Fondasi sains; NEL Discovery.
 Tema kosakata: tubuh, indra. Model latihan: 8, 1. Layar pelajaran: kenalan, kata, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4679,7 +4679,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -4693,7 +4693,7 @@
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
@@ -4767,7 +4767,7 @@
       <c r="S41" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-02 · Pra-TK · Sains · Hewan di sekitarku
+UNIT P-SA-02 · PAUD · Sains · Hewan di sekitarku
 Tujuan: Nama, suara, dan tempat hidup hewan. Rujukan: CP Fondasi sains.
 Tema kosakata: hewan peliharaan, ternak. Model latihan: 1, 7, 14. Layar pelajaran: kata, bunyi.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4778,7 +4778,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
@@ -4866,7 +4866,7 @@
       <c r="S42" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-03 · Pra-TK · Sains · Tumbuhan dan buah
+UNIT P-SA-03 · PAUD · Sains · Tumbuhan dan buah
 Tujuan: Bagian tumbuhan sederhana, buah lokal. Rujukan: CP Fondasi sains.
 Tema kosakata: buah, sayur, tanaman. Model latihan: 1, 7. Layar pelajaran: kata, cerita.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4877,7 +4877,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -4891,7 +4891,7 @@
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -4965,7 +4965,7 @@
       <c r="S43" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-04 · Pra-TK · Sains · Panas dan dingin
+UNIT P-SA-04 · PAUD · Sains · Panas dan dingin
 Tujuan: Merasakan suhu benda. Rujukan: CP Fondasi sains.
 Tema kosakata: dapur, minuman, alam. Model latihan: 7, 1. Layar pelajaran: kenalan, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -4976,7 +4976,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
@@ -5064,7 +5064,7 @@
       <c r="S44" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-05 · Pra-TK · Sains · Cuaca hari ini
+UNIT P-SA-05 · PAUD · Sains · Cuaca hari ini
 Tujuan: Cerah, hujan, berawan, berangin. Rujukan: CP Fondasi sains.
 Tema kosakata: cuaca, pakaian. Model latihan: 1, 8. Layar pelajaran: kata, cerita.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -5075,7 +5075,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -5163,7 +5163,7 @@
       <c r="S45" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-06 · Pra-TK · Sains · Siang dan malam
+UNIT P-SA-06 · PAUD · Sains · Siang dan malam
 Tujuan: Matahari, bulan, bintang. Rujukan: CP Fondasi sains.
 Tema kosakata: langit. Model latihan: 7, 1. Layar pelajaran: kata, cerita.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -5174,7 +5174,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5188,7 +5188,7 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
@@ -5262,7 +5262,7 @@
       <c r="S46" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-07 · Pra-TK · Sains · Tenggelam dan terapung
+UNIT P-SA-07 · PAUD · Sains · Tenggelam dan terapung
 Tujuan: Menduga lalu mengamati. Rujukan: NEL Discovery (inquiry).
 Tema kosakata: benda rumah. Model latihan: 7, 1. Layar pelajaran: cerita, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -5273,7 +5273,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
@@ -5361,7 +5361,7 @@
       <c r="S47" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-08 · Pra-TK · Sains · Air, es, dan uap
+UNIT P-SA-08 · PAUD · Sains · Air, es, dan uap
 Tujuan: Benda bisa berubah wujud. Rujukan: CP Fondasi sains.
 Tema kosakata: dapur, alam. Model latihan: 6, 7. Layar pelajaran: cerita, kata.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -5372,7 +5372,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -5460,7 +5460,7 @@
       <c r="S48" s="6" t="inlineStr">
         <is>
           <t>Kamu penulis konten Udakids (aplikasi belajar anak 4–7 tahun, Indonesia).
-UNIT P-SA-09 · Pra-TK · Sains · Bersih dan sehat
+UNIT P-SA-09 · PAUD · Sains · Bersih dan sehat
 Tujuan: Cuci tangan, sikat gigi, buang sampah. Rujukan: CP Fondasi (jati diri, kesehatan).
 Tema kosakata: kamar mandi, kegiatan. Model latihan: 6, 15. Layar pelajaran: cerita, coba.
 ATURAN WAJIB: bahasa Indonesia sederhana (English: perintah Indonesia, kata target English British); kalimat pendek;
@@ -5471,7 +5471,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.prek.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "prek", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5570,7 +5570,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5669,7 +5669,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5768,7 +5768,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5867,7 +5867,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -5966,7 +5966,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6065,7 +6065,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6164,7 +6164,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6263,7 +6263,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6362,7 +6362,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6461,7 +6461,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6560,7 +6560,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6659,7 +6659,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -6857,7 +6857,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -7253,7 +7253,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -7352,7 +7352,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -7649,7 +7649,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -8342,7 +8342,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "math.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "math", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -8441,7 +8441,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -8540,7 +8540,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -8639,7 +8639,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -8837,7 +8837,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -8936,7 +8936,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -9134,7 +9134,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -9233,7 +9233,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -9332,7 +9332,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -9431,7 +9431,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -9530,7 +9530,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -9728,7 +9728,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -9827,7 +9827,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11015,7 +11015,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11114,7 +11114,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.tk.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "tk", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11213,7 +11213,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11312,7 +11312,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11411,7 +11411,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11510,7 +11510,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11609,7 +11609,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11708,7 +11708,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11807,7 +11807,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -11906,7 +11906,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -12005,7 +12005,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -12104,7 +12104,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -12203,7 +12203,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -12302,7 +12302,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "literasi.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "literasi", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -13787,7 +13787,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -13886,7 +13886,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -13985,7 +13985,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -14084,7 +14084,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -14183,7 +14183,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -14282,7 +14282,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -14381,7 +14381,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -14480,7 +14480,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -14579,7 +14579,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -14678,7 +14678,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "english.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "english", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -16262,7 +16262,7 @@
 kenalan, bunyi, kata, gabung, cerita, coba, ingat. Setiap layar: "jenis", "teks" (≤ 120 huruf), "suara" (kalimat
 yang dibacakan), "gambar" (daftar id kata benda dari kamus, huruf kecil, tanpa spasi), dan untuk "kata" isi
 "sukuKata" (mis. "a-pel"). Layar terakhir "ingat".
-BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk Pra-TK/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
+BAGIAN B (soal): buat 10 file skill JSON (Level 1–10, mudah ke sulit, Level 10 tantangan gabungan) format Udakids: id "sains.sd1.&lt;kode&gt;&lt;n&gt;.&lt;slug&gt;", domain "sains", grade "sd1", family "manual" (atau family lain yang sudah ada), tier "basic" untuk PAUD/TK. Setiap level minimal 24 soal unik, 3–4 pilihan, satu jawaban benar, pengecoh dari miskonsepsi umum, setiap soal punya "say" (dibacakan), "reteach", dan "source". Gunakan hanya interaksi yang sudah ada (pick-one, tap-all, order, group, match, build, number-line, number-input).
 BAGIAN C (gambar): daftar kata benda baru yang butuh gambar, format "id | kata Indonesia | kata Inggris | tema".
 Keluarkan hanya JSON untuk A dan B, lalu daftar C.</t>
         </is>
@@ -16357,7 +16357,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16366,23 +16366,23 @@
         </is>
       </c>
       <c r="C2">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Baca Tulis")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Baca Tulis")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$I:$I,"BARU*")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$I:$I,"BARU*")</f>
         <v/>
       </c>
       <c r="E2">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$N:$N,"Draf")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$N:$N,"Draf")</f>
         <v/>
       </c>
       <c r="F2">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$N:$N,"Review")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$N:$N,"Review")</f>
         <v/>
       </c>
       <c r="G2">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$N:$N,"Terbit")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Baca Tulis",'Menu Belajar'!$N:$N,"Terbit")</f>
         <v/>
       </c>
       <c r="H2" s="11">
@@ -16393,7 +16393,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16402,23 +16402,23 @@
         </is>
       </c>
       <c r="C3">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Berhitung")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Berhitung")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$I:$I,"BARU*")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$I:$I,"BARU*")</f>
         <v/>
       </c>
       <c r="E3">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$N:$N,"Draf")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$N:$N,"Draf")</f>
         <v/>
       </c>
       <c r="F3">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$N:$N,"Review")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$N:$N,"Review")</f>
         <v/>
       </c>
       <c r="G3">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$N:$N,"Terbit")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Berhitung",'Menu Belajar'!$N:$N,"Terbit")</f>
         <v/>
       </c>
       <c r="H3" s="11">
@@ -16429,7 +16429,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16438,23 +16438,23 @@
         </is>
       </c>
       <c r="C4">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"English")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"English")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$I:$I,"BARU*")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$I:$I,"BARU*")</f>
         <v/>
       </c>
       <c r="E4">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$N:$N,"Draf")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$N:$N,"Draf")</f>
         <v/>
       </c>
       <c r="F4">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$N:$N,"Review")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$N:$N,"Review")</f>
         <v/>
       </c>
       <c r="G4">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$N:$N,"Terbit")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"English",'Menu Belajar'!$N:$N,"Terbit")</f>
         <v/>
       </c>
       <c r="H4" s="11">
@@ -16465,7 +16465,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pra-TK</t>
+          <t>PAUD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -16474,23 +16474,23 @@
         </is>
       </c>
       <c r="C5">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Sains")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Sains")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$I:$I,"BARU*")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$I:$I,"BARU*")</f>
         <v/>
       </c>
       <c r="E5">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$N:$N,"Draf")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$N:$N,"Draf")</f>
         <v/>
       </c>
       <c r="F5">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$N:$N,"Review")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$N:$N,"Review")</f>
         <v/>
       </c>
       <c r="G5">
-        <f>COUNTIFS('Menu Belajar'!$B:$B,"Pra-TK",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$N:$N,"Terbit")</f>
+        <f>COUNTIFS('Menu Belajar'!$B:$B,"PAUD",'Menu Belajar'!$C:$C,"Sains",'Menu Belajar'!$N:$N,"Terbit")</f>
         <v/>
       </c>
       <c r="H5" s="11">

</xml_diff>